<commit_message>
Implement anti-cheating measures: add tab switch detection and disable copy/paste functionality during exam
</commit_message>
<xml_diff>
--- a/JAMB Slips.xlsx
+++ b/JAMB Slips.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Documents\JAMB_App\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{83619551-0FA8-476C-B62C-4865FF3C8C98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DD73715-23C1-41DB-9B44-E5AEDC8A0852}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="732" yWindow="732" windowWidth="17280" windowHeight="9420" xr2:uid="{6CD54D3B-EF31-4377-8F6B-04DD1C271DA9}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{6CD54D3B-EF31-4377-8F6B-04DD1C271DA9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -642,10 +642,17 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -671,8 +678,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1011,594 +1019,594 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1">
+      <c r="B1" s="1">
         <v>8249</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="1">
         <v>1938</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="1">
         <v>5721</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+      <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="1">
         <v>3046</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+      <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="1">
         <v>9182</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+      <c r="A6" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="1">
         <v>4735</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+      <c r="A7" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B7">
+      <c r="B7" s="1">
         <v>6290</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
+      <c r="A8" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B8">
+      <c r="B8" s="1">
         <v>1584</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
+      <c r="A9" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B9">
+      <c r="B9" s="1">
         <v>8407</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
+      <c r="A10" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B10">
+      <c r="B10" s="1">
         <v>2613</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
+      <c r="A11" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B11">
+      <c r="B11" s="1">
         <v>9350</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
+      <c r="A12" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B12">
+      <c r="B12" s="1">
         <v>4827</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
+      <c r="A13" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B13">
+      <c r="B13" s="1">
         <v>7164</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
+      <c r="A14" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B14">
+      <c r="B14" s="1">
         <v>3592</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
+      <c r="A15" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B15">
+      <c r="B15" s="1">
         <v>6048</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
+      <c r="A16" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B16">
+      <c r="B16" s="1">
         <v>2915</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
+      <c r="A17" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B17">
+      <c r="B17" s="1">
         <v>8371</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
+      <c r="A18" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B18">
+      <c r="B18" s="1">
         <v>5409</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
+      <c r="A19" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B19">
+      <c r="B19" s="1">
         <v>1726</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
+      <c r="A20" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B20">
+      <c r="B20" s="1">
         <v>9583</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
+      <c r="A21" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B21">
+      <c r="B21" s="1">
         <v>3640</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
+      <c r="A22" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B22">
+      <c r="B22" s="1">
         <v>8195</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
+      <c r="A23" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B23">
+      <c r="B23" s="1">
         <v>4251</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
+      <c r="A24" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B24">
+      <c r="B24" s="1">
         <v>7038</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
+      <c r="A25" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B25">
+      <c r="B25" s="1">
         <v>2584</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
+      <c r="A26" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B26">
+      <c r="B26" s="1">
         <v>6917</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
+      <c r="A27" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B27">
+      <c r="B27" s="1">
         <v>1472</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
+      <c r="A28" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B28">
+      <c r="B28" s="1">
         <v>9820</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
+      <c r="A29" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B29">
+      <c r="B29" s="1">
         <v>5364</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A30" t="s">
+      <c r="A30" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B30">
+      <c r="B30" s="1">
         <v>3719</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A31" t="s">
+      <c r="A31" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B31">
+      <c r="B31" s="1">
         <v>8056</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A32" t="s">
+      <c r="A32" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B32">
+      <c r="B32" s="1">
         <v>2491</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A33" t="s">
+      <c r="A33" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B33">
+      <c r="B33" s="1">
         <v>6835</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A34" t="s">
+      <c r="A34" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B34">
+      <c r="B34" s="1">
         <v>1270</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A35" t="s">
+      <c r="A35" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B35">
+      <c r="B35" s="1">
         <v>9643</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A36" t="s">
+      <c r="A36" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B36">
+      <c r="B36" s="1">
         <v>5187</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A37" t="s">
+      <c r="A37" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B37">
+      <c r="B37" s="1">
         <v>7529</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A38" t="s">
+      <c r="A38" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B38">
+      <c r="B38" s="1">
         <v>3964</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A39" t="s">
+      <c r="A39" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B39">
+      <c r="B39" s="1">
         <v>8410</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A40" t="s">
+      <c r="A40" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B40">
+      <c r="B40" s="1">
         <v>4058</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A41" t="s">
+      <c r="A41" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B41">
+      <c r="B41" s="1">
         <v>6392</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A42" t="s">
+      <c r="A42" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B42">
+      <c r="B42" s="1">
         <v>1847</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A43" t="s">
+      <c r="A43" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B43">
+      <c r="B43" s="1">
         <v>9275</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A44" t="s">
+      <c r="A44" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="B44">
+      <c r="B44" s="1">
         <v>5610</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A45" t="s">
+      <c r="A45" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B45">
+      <c r="B45" s="1">
         <v>3154</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A46" t="s">
+      <c r="A46" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="B46">
+      <c r="B46" s="1">
         <v>7489</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A47" t="s">
+      <c r="A47" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B47">
+      <c r="B47" s="1">
         <v>2836</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A48" t="s">
+      <c r="A48" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="B48">
+      <c r="B48" s="1">
         <v>8571</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A49" t="s">
+      <c r="A49" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B49">
+      <c r="B49" s="1">
         <v>4915</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A50" t="s">
+      <c r="A50" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="B50">
+      <c r="B50" s="1">
         <v>6028</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A51" t="s">
+      <c r="A51" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B51">
+      <c r="B51" s="1">
         <v>1369</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A52" t="s">
+      <c r="A52" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="B52">
+      <c r="B52" s="1">
         <v>9704</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A53" t="s">
+      <c r="A53" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B53">
+      <c r="B53" s="1">
         <v>5248</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A54" t="s">
+      <c r="A54" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B54">
+      <c r="B54" s="1">
         <v>3681</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A55" t="s">
+      <c r="A55" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B55">
+      <c r="B55" s="1">
         <v>8125</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A56" t="s">
+      <c r="A56" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="B56">
+      <c r="B56" s="1">
         <v>2569</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A57" t="s">
+      <c r="A57" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B57">
+      <c r="B57" s="1">
         <v>7914</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A58" t="s">
+      <c r="A58" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="B58">
+      <c r="B58" s="1">
         <v>4350</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A59" t="s">
+      <c r="A59" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B59">
+      <c r="B59" s="1">
         <v>6782</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A60" t="s">
+      <c r="A60" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="B60">
+      <c r="B60" s="1">
         <v>1027</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A61" t="s">
+      <c r="A61" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="B61">
+      <c r="B61" s="1">
         <v>9456</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A62" t="s">
+      <c r="A62" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="B62">
+      <c r="B62" s="1">
         <v>5891</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A63" t="s">
+      <c r="A63" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="B63">
+      <c r="B63" s="1">
         <v>3247</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A64" t="s">
+      <c r="A64" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="B64">
+      <c r="B64" s="1">
         <v>8630</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A65" t="s">
+      <c r="A65" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="B65">
+      <c r="B65" s="1">
         <v>4075</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A66" t="s">
+      <c r="A66" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="B66">
+      <c r="B66" s="1">
         <v>7518</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A67" t="s">
+      <c r="A67" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="B67">
+      <c r="B67" s="1">
         <v>2953</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A68" t="s">
+      <c r="A68" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="B68">
+      <c r="B68" s="1">
         <v>6492</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A69" t="s">
+      <c r="A69" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="B69">
+      <c r="B69" s="1">
         <v>1836</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A70" t="s">
+      <c r="A70" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="B70">
+      <c r="B70" s="1">
         <v>9170</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A71" t="s">
+      <c r="A71" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B71">
+      <c r="B71" s="1">
         <v>5714</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A72" t="s">
+      <c r="A72" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="B72">
+      <c r="B72" s="1">
         <v>3059</v>
       </c>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A73" t="s">
+      <c r="A73" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="B73">
+      <c r="B73" s="1">
         <v>8592</v>
       </c>
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A74" t="s">
+      <c r="A74" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="B74">
+      <c r="B74" s="1">
         <v>4937</v>
       </c>
     </row>

</xml_diff>